<commit_message>
Complete six professor reports and repair first-week comparison tables
</commit_message>
<xml_diff>
--- a/results/six_week_reports_20261028/report_01_CN距離容差與Solver.xlsx
+++ b/results/six_week_reports_20261028/report_01_CN距離容差與Solver.xlsx
@@ -12,9 +12,9 @@
     <sheet name="精度時間與成對比較" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">四組結果比較!$A$1:$H$73</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">精度時間與成對比較!$A$1:$H$52</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">設定與說明!$A$1:$H$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">四組結果比較!$A$1:$H$76</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">精度時間與成對比較!$A$1:$H$79</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">設定與說明!$A$1:$H$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">四組結果比較!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">精度時間與成對比較!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">設定與說明!$1:$3</definedName>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="150">
   <si>
     <t>第1次｜CN距離容差與Solver</t>
   </si>
@@ -252,6 +252,75 @@
     <t>論文TableI的ETH e_p=15.3427cm，Tongji Plot1～4=5.2558/11.4808/4.8756/4.3560cm，各報100%；分母與成功門檻待補。四組本地控制實驗不是作者程式重跑；目前結果不支持「這兩項改動在所有場景都改善」。</t>
   </si>
   <si>
+    <t>原論文與本地四組：只列本週重要設定</t>
+  </si>
+  <si>
+    <t>原論文</t>
+  </si>
+  <si>
+    <t>本地修改前</t>
+  </si>
+  <si>
+    <t>本地修改後</t>
+  </si>
+  <si>
+    <t>不是成功門檻或voxel尺寸</t>
+  </si>
+  <si>
+    <t>剛體Solver</t>
+  </si>
+  <si>
+    <t>Euclidean transform；細節未交代</t>
+  </si>
+  <si>
+    <t>論文未說明，不把SVD稱作作者原始實作</t>
+  </si>
+  <si>
+    <t>新增弱配對補救</t>
+  </si>
+  <si>
+    <t>未描述本地evidence recovery</t>
+  </si>
+  <si>
+    <t>論文本身的triangle fallback仍在；與新增補救不同</t>
+  </si>
+  <si>
+    <t>N／w／Thscore</t>
+  </si>
+  <si>
+    <t>183／10／40</t>
+  </si>
+  <si>
+    <t>三項固定；沒有新增第三個實驗變數</t>
+  </si>
+  <si>
+    <t>論文時間與缺值原因：只作報告值參考</t>
+  </si>
+  <si>
+    <t>論文matching ms</t>
+  </si>
+  <si>
+    <t>論文total s</t>
+  </si>
+  <si>
+    <t>論文e_R／e_t</t>
+  </si>
+  <si>
+    <t>論文成功分母／門檻</t>
+  </si>
+  <si>
+    <t>時間可比性</t>
+  </si>
+  <si>
+    <t>未單獨報告；Table I用e_p</t>
+  </si>
+  <si>
+    <t>待補：本文未明確交代</t>
+  </si>
+  <si>
+    <t>i7-9700F 3GHz；實際threads未交代；本地計時範圍不同，不算加速比</t>
+  </si>
+  <si>
     <t>數據來源與比較限制</t>
   </si>
   <si>
@@ -379,6 +448,33 @@
   </si>
   <si>
     <t>ETH-tree；10cm固定；SVD→RANSAC</t>
+  </si>
+  <si>
+    <t>四組直接對照論文與修改前5cm/SVD；誤差下降率正值為降低、負值為變大</t>
+  </si>
+  <si>
+    <t>本地e_p cm</t>
+  </si>
+  <si>
+    <t>vs論文誤差下降率</t>
+  </si>
+  <si>
+    <t>vs修改前誤差下降率</t>
+  </si>
+  <si>
+    <t>vs論文成功率 pp</t>
+  </si>
+  <si>
+    <t>vs修改前成功率 pp</t>
+  </si>
+  <si>
+    <t>不可比：本地缺變換；有限N見前表</t>
+  </si>
+  <si>
+    <t>不可比：前後有限案例集合不同</t>
+  </si>
+  <si>
+    <t>vs論文是報告值的算術差異，並非同門檻／同配對的公平重跑。論文e_R/e_t未單獨報告、成功分母與門檻待補；不能由e_p推算。缺變換不是漏做實驗，也不能填0；前後有限集合不同請看共同成功對照。時間範圍不同不列下降率。</t>
   </si>
 </sst>
 </file>
@@ -463,7 +559,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -478,49 +574,52 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="172" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="173" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="174" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="175" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1286,14 +1385,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>752475</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1316,13 +1415,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>752475</xdr:colOff>
-      <xdr:row>67</xdr:row>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>69</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1637,11 +1736,8 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" customWidth="1"/>
-    <col min="3" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="7" width="20.7109375" customWidth="1"/>
-    <col min="8" max="8" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="8" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1">
@@ -2164,7 +2260,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.7109375" customWidth="1"/>
@@ -2237,7 +2333,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="45" customHeight="1">
+    <row r="7" spans="1:8" ht="60" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>28</v>
       </c>
@@ -2279,7 +2375,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="45" customHeight="1">
+    <row r="10" spans="1:8" ht="78" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>39</v>
       </c>
@@ -2341,13 +2437,13 @@
       <c r="C15" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F15" s="19">
+      <c r="F15" s="20">
         <f>(100/100-100/100)*100</f>
         <v>0.0</v>
       </c>
@@ -2368,13 +2464,13 @@
       <c r="C16" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F16" s="19">
+      <c r="F16" s="20">
         <f>(100/100-100/100)*100</f>
         <v>0.0</v>
       </c>
@@ -2395,13 +2491,13 @@
       <c r="C17" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="20">
         <f>(100/100-100/100)*100</f>
         <v>0.0</v>
       </c>
@@ -2422,13 +2518,13 @@
       <c r="C18" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F18" s="19">
+      <c r="F18" s="20">
         <f>(100/100-100/100)*100</f>
         <v>0.0</v>
       </c>
@@ -2449,13 +2545,13 @@
       <c r="C19" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="19">
+      <c r="F19" s="20">
         <f>(37/100-33/100)*100</f>
         <v>3.9999999999999982</v>
       </c>
@@ -2476,13 +2572,13 @@
       <c r="C20" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="20">
         <f>(34/100-28/100)*100</f>
         <v>6.0</v>
       </c>
@@ -2503,13 +2599,13 @@
       <c r="C21" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="20">
         <f>(28/100-33/100)*100</f>
         <v>-4.999999999999999</v>
       </c>
@@ -2530,13 +2626,13 @@
       <c r="C22" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="F22" s="19">
+      <c r="F22" s="20">
         <f>(34/100-37/100)*100</f>
         <v>-2.9999999999999973</v>
       </c>
@@ -2557,13 +2653,13 @@
       <c r="C23" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F23" s="19">
+      <c r="F23" s="20">
         <f>(100/100-100/100)*100</f>
         <v>0.0</v>
       </c>
@@ -2584,13 +2680,13 @@
       <c r="C24" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="20">
         <f>(100/100-100/100)*100</f>
         <v>0.0</v>
       </c>
@@ -2611,13 +2707,13 @@
       <c r="C25" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F25" s="19">
+      <c r="F25" s="20">
         <f>(100/100-100/100)*100</f>
         <v>0.0</v>
       </c>
@@ -2638,13 +2734,13 @@
       <c r="C26" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F26" s="19">
+      <c r="F26" s="20">
         <f>(100/100-100/100)*100</f>
         <v>0.0</v>
       </c>
@@ -2665,13 +2761,13 @@
       <c r="C27" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="F27" s="19">
+      <c r="F27" s="20">
         <f>(69/100-76/100)*100</f>
         <v>-7.000000000000006</v>
       </c>
@@ -2692,13 +2788,13 @@
       <c r="C28" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="F28" s="19">
+      <c r="F28" s="20">
         <f>(70/100-76/100)*100</f>
         <v>-6.000000000000005</v>
       </c>
@@ -2719,13 +2815,13 @@
       <c r="C29" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="F29" s="19">
+      <c r="F29" s="20">
         <f>(76/100-76/100)*100</f>
         <v>0.0</v>
       </c>
@@ -2746,13 +2842,13 @@
       <c r="C30" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="F30" s="19">
+      <c r="F30" s="20">
         <f>(70/100-69/100)*100</f>
         <v>1.0000000000000009</v>
       </c>
@@ -2773,13 +2869,13 @@
       <c r="C31" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="F31" s="19">
+      <c r="F31" s="20">
         <f>(138/150-114/150)*100</f>
         <v>16.000000000000004</v>
       </c>
@@ -2800,13 +2896,13 @@
       <c r="C32" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F32" s="19">
+      <c r="F32" s="20">
         <f>(144/150-121/150)*100</f>
         <v>15.333333333333332</v>
       </c>
@@ -2827,13 +2923,13 @@
       <c r="C33" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="F33" s="19">
+      <c r="F33" s="20">
         <f>(121/150-114/150)*100</f>
         <v>4.666666666666663</v>
       </c>
@@ -2854,13 +2950,13 @@
       <c r="C34" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="F34" s="19">
+      <c r="F34" s="20">
         <f>(144/150-138/150)*100</f>
         <v>3.9999999999999925</v>
       </c>
@@ -2919,44 +3015,273 @@
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
     </row>
-    <row r="44" spans="1:8" ht="38" customHeight="1">
-      <c r="A44" s="2" t="s">
+    <row r="44" spans="1:8" ht="40" customHeight="1">
+      <c r="A44" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="2"/>
-    </row>
-    <row r="45" spans="1:8" ht="38" customHeight="1">
-      <c r="A45" s="2" t="s">
+      <c r="C44" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-    </row>
-    <row r="46" spans="1:8" ht="52" customHeight="1">
-      <c r="A46" s="2" t="s">
+      <c r="D44" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
+      <c r="E44" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="45" customHeight="1">
+      <c r="A45" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="60" customHeight="1">
+      <c r="A46" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="78" customHeight="1">
+      <c r="A47" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="60" customHeight="1">
+      <c r="A48" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="28" customHeight="1">
+      <c r="A51" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+    </row>
+    <row r="52" spans="1:8" ht="40" customHeight="1">
+      <c r="A52" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="96" customHeight="1">
+      <c r="A53" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B53" s="7">
+        <v>20.718</v>
+      </c>
+      <c r="C53" s="7">
+        <v>11.657</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="96" customHeight="1">
+      <c r="A54" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B54" s="7">
+        <v>30.699</v>
+      </c>
+      <c r="C54" s="7">
+        <v>16.712</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="96" customHeight="1">
+      <c r="A55" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B55" s="7">
+        <v>4.5596</v>
+      </c>
+      <c r="C55" s="7">
+        <v>8.3584</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="96" customHeight="1">
+      <c r="A56" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B56" s="7">
+        <v>19.522</v>
+      </c>
+      <c r="C56" s="7">
+        <v>9.451599999999999</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="96" customHeight="1">
+      <c r="A57" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B57" s="7">
+        <v>3.0405</v>
+      </c>
+      <c r="C57" s="7">
+        <v>8.699199999999999</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="28" customHeight="1">
+      <c r="A60" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B60" s="3"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+    </row>
+    <row r="61" spans="1:8" ht="38" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+    </row>
+    <row r="62" spans="1:8" ht="38" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
+      <c r="F62" s="2"/>
+      <c r="G62" s="2"/>
+      <c r="H62" s="2"/>
+    </row>
+    <row r="63" spans="1:8" ht="52" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+      <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
@@ -2966,9 +3291,11 @@
     <mergeCell ref="A39:H39"/>
     <mergeCell ref="A41:H41"/>
     <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A60:H60"/>
+    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A63:H63"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" fitToHeight="0" orientation="landscape"/>
@@ -2984,7 +3311,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.7109375" customWidth="1"/>
@@ -3033,7 +3360,7 @@
     </row>
     <row r="5" spans="1:8" ht="28" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -3048,25 +3375,25 @@
         <v>44</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="45" customHeight="1">
@@ -3091,7 +3418,7 @@
       <c r="G7" s="7">
         <v>24.15578572</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="19" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3117,7 +3444,7 @@
       <c r="G8" s="7">
         <v>26.64002224</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="19" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3143,7 +3470,7 @@
       <c r="G9" s="7">
         <v>25.05820484</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="19" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3169,7 +3496,7 @@
       <c r="G10" s="7">
         <v>27.09175617</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="19" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3195,7 +3522,7 @@
       <c r="G11" s="7">
         <v>66.57111264</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="19" t="s">
         <v>61</v>
       </c>
     </row>
@@ -3221,7 +3548,7 @@
       <c r="G12" s="7">
         <v>69.86197643</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="19" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3247,7 +3574,7 @@
       <c r="G13" s="7">
         <v>56.89672242</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="19" t="s">
         <v>62</v>
       </c>
     </row>
@@ -3273,7 +3600,7 @@
       <c r="G14" s="7">
         <v>61.17425436</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="19" t="s">
         <v>64</v>
       </c>
     </row>
@@ -3299,7 +3626,7 @@
       <c r="G15" s="7">
         <v>6.04477203</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="19" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3325,7 +3652,7 @@
       <c r="G16" s="7">
         <v>7.29747341</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="19" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3351,7 +3678,7 @@
       <c r="G17" s="7">
         <v>6.71977696</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="H17" s="19" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3377,7 +3704,7 @@
       <c r="G18" s="7">
         <v>8.32219845</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="19" t="s">
         <v>54</v>
       </c>
     </row>
@@ -3403,7 +3730,7 @@
       <c r="G19" s="7">
         <v>6.01696067</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="19" t="s">
         <v>65</v>
       </c>
     </row>
@@ -3429,7 +3756,7 @@
       <c r="G20" s="7">
         <v>6.60275653</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="H20" s="19" t="s">
         <v>65</v>
       </c>
     </row>
@@ -3455,7 +3782,7 @@
       <c r="G21" s="7">
         <v>6.25656317</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="H21" s="19" t="s">
         <v>66</v>
       </c>
     </row>
@@ -3481,7 +3808,7 @@
       <c r="G22" s="7">
         <v>7.46682261</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="19" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3507,7 +3834,7 @@
       <c r="G23" s="7">
         <v>2.37528938</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="19" t="s">
         <v>68</v>
       </c>
     </row>
@@ -3533,7 +3860,7 @@
       <c r="G24" s="7">
         <v>2.804647686666667</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="19" t="s">
         <v>70</v>
       </c>
     </row>
@@ -3559,7 +3886,7 @@
       <c r="G25" s="7">
         <v>2.443533233333333</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="19" t="s">
         <v>69</v>
       </c>
     </row>
@@ -3585,13 +3912,13 @@
       <c r="G26" s="7">
         <v>3.046398766666667</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="19" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="42" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -3603,7 +3930,7 @@
     </row>
     <row r="31" spans="1:8" ht="28" customHeight="1">
       <c r="A31" s="3" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -3615,33 +3942,33 @@
     </row>
     <row r="32" spans="1:8" ht="40" customHeight="1">
       <c r="A32" s="3" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="45" customHeight="1">
       <c r="A33" s="4" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="B33" s="4">
         <v>0</v>
@@ -3663,12 +3990,12 @@
         <v>-0.050806072728931416</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="45" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="B34" s="4">
         <v>0</v>
@@ -3690,12 +4017,12 @@
         <v>-0.012503432830581362</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="45" customHeight="1">
       <c r="A35" s="4" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="B35" s="4">
         <v>0</v>
@@ -3717,12 +4044,12 @@
         <v>-0.02353700175334276</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="45" customHeight="1">
       <c r="A36" s="4" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="B36" s="4">
         <v>0</v>
@@ -3744,12 +4071,12 @@
         <v>0.013771660823170901</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="45" customHeight="1">
       <c r="A37" s="4" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="B37" s="4">
         <v>8</v>
@@ -3771,12 +4098,12 @@
         <v>0.02259266003983248</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="45" customHeight="1">
       <c r="A38" s="4" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="B38" s="4">
         <v>9</v>
@@ -3798,12 +4125,12 @@
         <v>0.007403011167682776</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="45" customHeight="1">
       <c r="A39" s="4" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="B39" s="4">
         <v>7</v>
@@ -3825,12 +4152,12 @@
         <v>0.06844395066047179</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="45" customHeight="1">
       <c r="A40" s="4" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="B40" s="4">
         <v>9</v>
@@ -3852,12 +4179,12 @@
         <v>0.04548307953652312</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="45" customHeight="1">
       <c r="A41" s="4" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="B41" s="4">
         <v>0</v>
@@ -3879,12 +4206,12 @@
         <v>0.07118981449234645</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="45" customHeight="1">
       <c r="A42" s="4" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="B42" s="4">
         <v>0</v>
@@ -3906,12 +4233,12 @@
         <v>0.07370363074739225</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="45" customHeight="1">
       <c r="A43" s="4" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="B43" s="4">
         <v>0</v>
@@ -3933,12 +4260,12 @@
         <v>0.015748564299178053</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="45" customHeight="1">
       <c r="A44" s="4" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="B44" s="4">
         <v>0</v>
@@ -3960,12 +4287,12 @@
         <v>0.018412431789783346</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="45" customHeight="1">
       <c r="A45" s="4" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="B45" s="4">
         <v>6</v>
@@ -3987,12 +4314,12 @@
         <v>-0.015082134704163098</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="45" customHeight="1">
       <c r="A46" s="4" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="B46" s="4">
         <v>6</v>
@@ -4014,12 +4341,12 @@
         <v>-0.015241994755485188</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="45" customHeight="1">
       <c r="A47" s="4" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="B47" s="4">
         <v>0</v>
@@ -4041,12 +4368,12 @@
         <v>0.0</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="45" customHeight="1">
       <c r="A48" s="4" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="B48" s="4">
         <v>1</v>
@@ -4068,12 +4395,12 @@
         <v>0.0</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="45" customHeight="1">
       <c r="A49" s="4" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="B49" s="4">
         <v>28</v>
@@ -4095,12 +4422,12 @@
         <v>0.06822921201423354</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="45" customHeight="1">
       <c r="A50" s="4" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="B50" s="4">
         <v>25</v>
@@ -4122,12 +4449,12 @@
         <v>0.1282886319955973</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="45" customHeight="1">
       <c r="A51" s="4" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="B51" s="4">
         <v>7</v>
@@ -4149,12 +4476,12 @@
         <v>-0.004040251026809923</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="45" customHeight="1">
       <c r="A52" s="4" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="B52" s="4">
         <v>6</v>
@@ -4176,17 +4503,657 @@
         <v>0.08011103790036085</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>98</v>
-      </c>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="28" customHeight="1">
+      <c r="A55" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+    </row>
+    <row r="56" spans="1:8" ht="40" customHeight="1">
+      <c r="A56" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="45" customHeight="1">
+      <c r="A57" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" s="7">
+        <v>5.2558</v>
+      </c>
+      <c r="D57" s="7">
+        <v>16.81264811113</v>
+      </c>
+      <c r="E57" s="6">
+        <f>IF(AND(ISNUMBER(C57),ISNUMBER(D57),C57&lt;&gt;0),(C57-D57)/C57,"不可比")</f>
+        <v>-2.198875168600403</v>
+      </c>
+      <c r="F57" s="6">
+        <f>IF(AND(ISNUMBER(D57),16.81264811113&lt;&gt;0),(16.81264811113-D57)/16.81264811113,"不可比")</f>
+        <v>0.0</v>
+      </c>
+      <c r="G57" s="20">
+        <f>(100/100-1)*100</f>
+        <v>0.0</v>
+      </c>
+      <c r="H57" s="20">
+        <f>(100/100-100/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="45" customHeight="1">
+      <c r="A58" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C58" s="7">
+        <v>5.2558</v>
+      </c>
+      <c r="D58" s="7">
+        <v>17.2083674392</v>
+      </c>
+      <c r="E58" s="6">
+        <f>IF(AND(ISNUMBER(C58),ISNUMBER(D58),C58&lt;&gt;0),(C58-D58)/C58,"不可比")</f>
+        <v>-2.274167099052476</v>
+      </c>
+      <c r="F58" s="6">
+        <f>IF(AND(ISNUMBER(D58),16.81264811113&lt;&gt;0),(16.81264811113-D58)/16.81264811113,"不可比")</f>
+        <v>-0.02353700175334276</v>
+      </c>
+      <c r="G58" s="20">
+        <f>(100/100-1)*100</f>
+        <v>0.0</v>
+      </c>
+      <c r="H58" s="20">
+        <f>(100/100-100/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="45" customHeight="1">
+      <c r="A59" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" s="7">
+        <v>5.2558</v>
+      </c>
+      <c r="D59" s="7">
+        <v>17.66683273383</v>
+      </c>
+      <c r="E59" s="6">
+        <f>IF(AND(ISNUMBER(C59),ISNUMBER(D59),C59&lt;&gt;0),(C59-D59)/C59,"不可比")</f>
+        <v>-2.361397453067088</v>
+      </c>
+      <c r="F59" s="6">
+        <f>IF(AND(ISNUMBER(D59),16.81264811113&lt;&gt;0),(16.81264811113-D59)/16.81264811113,"不可比")</f>
+        <v>-0.050806072728931416</v>
+      </c>
+      <c r="G59" s="20">
+        <f>(100/100-1)*100</f>
+        <v>0.0</v>
+      </c>
+      <c r="H59" s="20">
+        <f>(100/100-100/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="45" customHeight="1">
+      <c r="A60" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="7">
+        <v>5.2558</v>
+      </c>
+      <c r="D60" s="7">
+        <v>17.4235311056</v>
+      </c>
+      <c r="E60" s="6">
+        <f>IF(AND(ISNUMBER(C60),ISNUMBER(D60),C60&lt;&gt;0),(C60-D60)/C60,"不可比")</f>
+        <v>-2.3151054274515777</v>
+      </c>
+      <c r="F60" s="6">
+        <f>IF(AND(ISNUMBER(D60),16.81264811113&lt;&gt;0),(16.81264811113-D60)/16.81264811113,"不可比")</f>
+        <v>-0.03633472790438032</v>
+      </c>
+      <c r="G60" s="20">
+        <f>(100/100-1)*100</f>
+        <v>0.0</v>
+      </c>
+      <c r="H60" s="20">
+        <f>(100/100-100/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="45" customHeight="1">
+      <c r="A61" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" s="7">
+        <v>11.4808</v>
+      </c>
+      <c r="D61" s="7">
+        <v>54.50497163930999</v>
+      </c>
+      <c r="E61" s="6">
+        <f>IF(AND(ISNUMBER(C61),ISNUMBER(D61),C61&lt;&gt;0),(C61-D61)/C61,"不可比")</f>
+        <v>-3.7474889937382407</v>
+      </c>
+      <c r="F61" s="6">
+        <f>IF(AND(ISNUMBER(D61),54.50497163930999&lt;&gt;0),(54.50497163930999-D61)/54.50497163930999,"不可比")</f>
+        <v>0.0</v>
+      </c>
+      <c r="G61" s="20">
+        <f>(33/100-1)*100</f>
+        <v>-67.0</v>
+      </c>
+      <c r="H61" s="20">
+        <f>(33/100-33/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="45" customHeight="1">
+      <c r="A62" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" s="7">
+        <v>11.4808</v>
+      </c>
+      <c r="D62" s="7">
+        <v>58.201283144</v>
+      </c>
+      <c r="E62" s="6">
+        <f>IF(AND(ISNUMBER(C62),ISNUMBER(D62),C62&lt;&gt;0),(C62-D62)/C62,"不可比")</f>
+        <v>-4.069444911852833</v>
+      </c>
+      <c r="F62" s="6">
+        <f>IF(AND(ISNUMBER(D62),54.50497163930999&lt;&gt;0),(54.50497163930999-D62)/54.50497163930999,"不可比")</f>
+        <v>-0.06781604307861266</v>
+      </c>
+      <c r="G62" s="20">
+        <f>(28/100-1)*100</f>
+        <v>-72.0</v>
+      </c>
+      <c r="H62" s="20">
+        <f>(28/100-33/100)*100</f>
+        <v>-4.999999999999999</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="45" customHeight="1">
+      <c r="A63" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C63" s="7">
+        <v>11.4808</v>
+      </c>
+      <c r="D63" s="7">
+        <v>47.25469538884</v>
+      </c>
+      <c r="E63" s="6">
+        <f>IF(AND(ISNUMBER(C63),ISNUMBER(D63),C63&lt;&gt;0),(C63-D63)/C63,"不可比")</f>
+        <v>-3.115975836948645</v>
+      </c>
+      <c r="F63" s="6">
+        <f>IF(AND(ISNUMBER(D63),54.50497163930999&lt;&gt;0),(54.50497163930999-D63)/54.50497163930999,"不可比")</f>
+        <v>0.13302045726120443</v>
+      </c>
+      <c r="G63" s="20">
+        <f>(37/100-1)*100</f>
+        <v>-63.0</v>
+      </c>
+      <c r="H63" s="20">
+        <f>(37/100-33/100)*100</f>
+        <v>3.9999999999999982</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" ht="45" customHeight="1">
+      <c r="A64" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C64" s="7">
+        <v>11.4808</v>
+      </c>
+      <c r="D64" s="7">
+        <v>50.90068114483</v>
+      </c>
+      <c r="E64" s="6">
+        <f>IF(AND(ISNUMBER(C64),ISNUMBER(D64),C64&lt;&gt;0),(C64-D64)/C64,"不可比")</f>
+        <v>-3.433548284512403</v>
+      </c>
+      <c r="F64" s="6">
+        <f>IF(AND(ISNUMBER(D64),54.50497163930999&lt;&gt;0),(54.50497163930999-D64)/54.50497163930999,"不可比")</f>
+        <v>0.06612773818747425</v>
+      </c>
+      <c r="G64" s="20">
+        <f>(34/100-1)*100</f>
+        <v>-65.99999999999999</v>
+      </c>
+      <c r="H64" s="20">
+        <f>(34/100-33/100)*100</f>
+        <v>1.0000000000000009</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" ht="45" customHeight="1">
+      <c r="A65" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C65" s="7">
+        <v>4.8756</v>
+      </c>
+      <c r="D65" s="7">
+        <v>5.376450884124</v>
+      </c>
+      <c r="E65" s="6">
+        <f>IF(AND(ISNUMBER(C65),ISNUMBER(D65),C65&lt;&gt;0),(C65-D65)/C65,"不可比")</f>
+        <v>-0.10272599969726795</v>
+      </c>
+      <c r="F65" s="6">
+        <f>IF(AND(ISNUMBER(D65),5.376450884124&lt;&gt;0),(5.376450884124-D65)/5.376450884124,"不可比")</f>
+        <v>0.0</v>
+      </c>
+      <c r="G65" s="20">
+        <f>(100/100-1)*100</f>
+        <v>0.0</v>
+      </c>
+      <c r="H65" s="20">
+        <f>(100/100-100/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="45" customHeight="1">
+      <c r="A66" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C66" s="7">
+        <v>4.8756</v>
+      </c>
+      <c r="D66" s="7">
+        <v>5.291779501674</v>
+      </c>
+      <c r="E66" s="6">
+        <f>IF(AND(ISNUMBER(C66),ISNUMBER(D66),C66&lt;&gt;0),(C66-D66)/C66,"不可比")</f>
+        <v>-0.08535964838666013</v>
+      </c>
+      <c r="F66" s="6">
+        <f>IF(AND(ISNUMBER(D66),5.376450884124&lt;&gt;0),(5.376450884124-D66)/5.376450884124,"不可比")</f>
+        <v>0.015748564299178053</v>
+      </c>
+      <c r="G66" s="20">
+        <f>(100/100-1)*100</f>
+        <v>0.0</v>
+      </c>
+      <c r="H66" s="20">
+        <f>(100/100-100/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="45" customHeight="1">
+      <c r="A67" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C67" s="7">
+        <v>4.8756</v>
+      </c>
+      <c r="D67" s="7">
+        <v>4.993702343056</v>
+      </c>
+      <c r="E67" s="6">
+        <f>IF(AND(ISNUMBER(C67),ISNUMBER(D67),C67&lt;&gt;0),(C67-D67)/C67,"不可比")</f>
+        <v>-0.024223140342932166</v>
+      </c>
+      <c r="F67" s="6">
+        <f>IF(AND(ISNUMBER(D67),5.376450884124&lt;&gt;0),(5.376450884124-D67)/5.376450884124,"不可比")</f>
+        <v>0.07118981449234645</v>
+      </c>
+      <c r="G67" s="20">
+        <f>(100/100-1)*100</f>
+        <v>0.0</v>
+      </c>
+      <c r="H67" s="20">
+        <f>(100/100-100/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="45" customHeight="1">
+      <c r="A68" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C68" s="7">
+        <v>4.8756</v>
+      </c>
+      <c r="D68" s="7">
+        <v>4.901756139286</v>
+      </c>
+      <c r="E68" s="6">
+        <f>IF(AND(ISNUMBER(C68),ISNUMBER(D68),C68&lt;&gt;0),(C68-D68)/C68,"不可比")</f>
+        <v>-0.005364701633850232</v>
+      </c>
+      <c r="F68" s="6">
+        <f>IF(AND(ISNUMBER(D68),5.376450884124&lt;&gt;0),(5.376450884124-D68)/5.376450884124,"不可比")</f>
+        <v>0.08829146867866212</v>
+      </c>
+      <c r="G68" s="20">
+        <f>(100/100-1)*100</f>
+        <v>0.0</v>
+      </c>
+      <c r="H68" s="20">
+        <f>(100/100-100/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="45" customHeight="1">
+      <c r="A69" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" s="7">
+        <v>4.356</v>
+      </c>
+      <c r="D69" s="7">
+        <v>123.2346789297831</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F69" s="6">
+        <f>IF(AND(ISNUMBER(D69),123.23467892978313&lt;&gt;0),(123.23467892978313-D69)/123.23467892978313,"不可比")</f>
+        <v>0.0</v>
+      </c>
+      <c r="G69" s="20">
+        <f>(76/100-1)*100</f>
+        <v>-24.0</v>
+      </c>
+      <c r="H69" s="20">
+        <f>(76/100-76/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="45" customHeight="1">
+      <c r="A70" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C70" s="7">
+        <v>4.356</v>
+      </c>
+      <c r="D70" s="7">
+        <v>123.2346789297831</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F70" s="6">
+        <f>IF(AND(ISNUMBER(D70),123.23467892978313&lt;&gt;0),(123.23467892978313-D70)/123.23467892978313,"不可比")</f>
+        <v>0.0</v>
+      </c>
+      <c r="G70" s="20">
+        <f>(76/100-1)*100</f>
+        <v>-24.0</v>
+      </c>
+      <c r="H70" s="20">
+        <f>(76/100-76/100)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" ht="45" customHeight="1">
+      <c r="A71" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C71" s="7">
+        <v>4.356</v>
+      </c>
+      <c r="D71" s="7">
+        <v>299.4917599032963</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G71" s="20">
+        <f>(69/100-1)*100</f>
+        <v>-31.000000000000007</v>
+      </c>
+      <c r="H71" s="20">
+        <f>(69/100-76/100)*100</f>
+        <v>-7.000000000000006</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" ht="45" customHeight="1">
+      <c r="A72" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C72" s="7">
+        <v>4.356</v>
+      </c>
+      <c r="D72" s="7">
+        <v>252.1680517323086</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G72" s="20">
+        <f>(70/100-1)*100</f>
+        <v>-30.000000000000004</v>
+      </c>
+      <c r="H72" s="20">
+        <f>(70/100-76/100)*100</f>
+        <v>-6.000000000000005</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" ht="45" customHeight="1">
+      <c r="A73" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C73" s="7">
+        <v>15.3427</v>
+      </c>
+      <c r="D73" s="7">
+        <v>12.62093021071654</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F73" s="6">
+        <f>IF(AND(ISNUMBER(D73),12.620930210716535&lt;&gt;0),(12.620930210716535-D73)/12.620930210716535,"不可比")</f>
+        <v>0.0</v>
+      </c>
+      <c r="G73" s="20">
+        <f>(114/150-1)*100</f>
+        <v>-24.0</v>
+      </c>
+      <c r="H73" s="20">
+        <f>(114/150-114/150)*100</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" ht="45" customHeight="1">
+      <c r="A74" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C74" s="7">
+        <v>15.3427</v>
+      </c>
+      <c r="D74" s="7">
+        <v>10.97050868271654</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F74" s="6">
+        <f>IF(AND(ISNUMBER(D74),12.620930210716535&lt;&gt;0),(12.620930210716535-D74)/12.620930210716535,"不可比")</f>
+        <v>0.13076861217397537</v>
+      </c>
+      <c r="G74" s="20">
+        <f>(121/150-1)*100</f>
+        <v>-19.333333333333336</v>
+      </c>
+      <c r="H74" s="20">
+        <f>(121/150-114/150)*100</f>
+        <v>4.666666666666663</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" ht="45" customHeight="1">
+      <c r="A75" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C75" s="7">
+        <v>15.3427</v>
+      </c>
+      <c r="D75" s="7">
+        <v>10.72940896452414</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G75" s="20">
+        <f>(138/150-1)*100</f>
+        <v>-7.9999999999999964</v>
+      </c>
+      <c r="H75" s="20">
+        <f>(138/150-114/150)*100</f>
+        <v>16.000000000000004</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" ht="45" customHeight="1">
+      <c r="A76" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C76" s="7">
+        <v>15.3427</v>
+      </c>
+      <c r="D76" s="7">
+        <v>9.095719413689656</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G76" s="20">
+        <f>(144/150-1)*100</f>
+        <v>-4.0000000000000036</v>
+      </c>
+      <c r="H76" s="20">
+        <f>(144/150-114/150)*100</f>
+        <v>19.999999999999996</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" ht="66" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B79" s="2"/>
+      <c r="C79" s="2"/>
+      <c r="D79" s="2"/>
+      <c r="E79" s="2"/>
+      <c r="F79" s="2"/>
+      <c r="G79" s="2"/>
+      <c r="H79" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A79:H79"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" fitToHeight="0" orientation="landscape"/>

</xml_diff>